<commit_message>
Compressor fix for crankcase flag errors
</commit_message>
<xml_diff>
--- a/input/Studies/MEET2/TankBatteryMassFlow.xlsx
+++ b/input/Studies/MEET2/TankBatteryMassFlow.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MEET2_main\input\Studies\MEET2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES\input\Studies\MEET2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3F5554-5737-4FFE-A2B0-0081A66CBFE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903FAEEC-A5B0-4F76-8345-B7616E546A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="937" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="937" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="245">
   <si>
     <t>Simulation Start Date</t>
   </si>
@@ -468,9 +468,6 @@
     <t>Well.json</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>ContinuousSeparator.json</t>
   </si>
   <si>
@@ -564,12 +561,6 @@
     <t>Blowdown Vent Component Count</t>
   </si>
   <si>
-    <t>Blowdown Vent MTTRMin</t>
-  </si>
-  <si>
-    <t>Blowdown Vent MTTRMax</t>
-  </si>
-  <si>
     <t>Blowdown Vent pLeak</t>
   </si>
   <si>
@@ -579,60 +570,30 @@
     <t>Common Single-Unit Vent Component Count</t>
   </si>
   <si>
-    <t>Common Single-Unit Vent MTTR Min</t>
-  </si>
-  <si>
-    <t>Common Single-Unit Vent MTTR Max</t>
-  </si>
-  <si>
     <t>Common Single-Unit Vent pLeak</t>
   </si>
   <si>
     <t>Seal Vent Component Count</t>
   </si>
   <si>
-    <t>Seal Vent MTTR Min</t>
-  </si>
-  <si>
-    <t>Seal Vent MTTR Max</t>
-  </si>
-  <si>
     <t>Seal Vent pLeak</t>
   </si>
   <si>
     <t>Seal Vent(Large Emitter) Component Count</t>
   </si>
   <si>
-    <t>Seal Vent(Large Emitter) MTTR Min</t>
-  </si>
-  <si>
-    <t>Seal Vent(Large Emitter) MTTR Max</t>
-  </si>
-  <si>
     <t>Seal Vent(Large Emitter) pLeak</t>
   </si>
   <si>
     <t>Compressor Starter Vent Component Count</t>
   </si>
   <si>
-    <t>Compressor Starter Vent MTTR Min</t>
-  </si>
-  <si>
-    <t>Compressor Starter Vent MTTR Max</t>
-  </si>
-  <si>
     <t>Compressor Starter Vent pLeak</t>
   </si>
   <si>
     <t>Common Single-unit Vent(Large Emitter) Component Count</t>
   </si>
   <si>
-    <t>Common Single-unit Vent(Large Emitter) MTTR Min</t>
-  </si>
-  <si>
-    <t>Common Single-unit Vent(Large Emitter) MTTR Max</t>
-  </si>
-  <si>
     <t>Common Single-unit Vent(Large Emitter) pLeak</t>
   </si>
   <si>
@@ -654,19 +615,7 @@
     <t>ts_compressor</t>
   </si>
   <si>
-    <t>4SRB</t>
-  </si>
-  <si>
-    <t>Common\EnginesFuelConsumpEq\4SRB\4SRB_400HP_G3408_Caterpillar.csv</t>
-  </si>
-  <si>
     <t>Centrifugal</t>
-  </si>
-  <si>
-    <t>Stage3</t>
-  </si>
-  <si>
-    <t>Well-Condensate.Stage1-Condensate.Stage2-Condensate.Stage3-Flash</t>
   </si>
   <si>
     <t>vrt</t>
@@ -795,9 +744,6 @@
     <t>Max Downstream Equipment Capacity [scfh]</t>
   </si>
   <si>
-    <t>gef_tank</t>
-  </si>
-  <si>
     <t>Lean Glycol Circulation Rate [gal/min]</t>
   </si>
   <si>
@@ -814,6 +760,63 @@
   </si>
   <si>
     <t>Tank Controlled [True, False]</t>
+  </si>
+  <si>
+    <t>ContinuousWells</t>
+  </si>
+  <si>
+    <t>wellpad_tanks</t>
+  </si>
+  <si>
+    <t>Crankcase Emissions Flag [TRUE, FALSE]</t>
+  </si>
+  <si>
+    <t>CCEE Ratio Distribution</t>
+  </si>
+  <si>
+    <t>Actuator Type [Gas, Air, Electric, Gas Mechanistic]</t>
+  </si>
+  <si>
+    <t>Blowdown Vent MTTRMin [days]</t>
+  </si>
+  <si>
+    <t>Blowdown Vent MTTRMax [days]</t>
+  </si>
+  <si>
+    <t>Common Single-Unit Vent MTTR Min [days]</t>
+  </si>
+  <si>
+    <t>Common Single-Unit Vent MTTR Max [days]</t>
+  </si>
+  <si>
+    <t>Seal Vent MTTR Min [days]</t>
+  </si>
+  <si>
+    <t>Seal Vent MTTR Max [days]</t>
+  </si>
+  <si>
+    <t>Seal Vent(Large Emitter) MTTR Min [days]</t>
+  </si>
+  <si>
+    <t>Seal Vent(Large Emitter) MTTR Max [days]</t>
+  </si>
+  <si>
+    <t>Compressor Starter Vent MTTR Min [days]</t>
+  </si>
+  <si>
+    <t>Compressor Starter Vent MTTR Max [days]</t>
+  </si>
+  <si>
+    <t>Common Single-unit Vent(Large Emitter) MTTR Min [days]</t>
+  </si>
+  <si>
+    <t>Common Single-unit Vent(Large Emitter) MTTR Max [days]</t>
+  </si>
+  <si>
+    <t>Turbine</t>
+  </si>
+  <si>
+    <t>EnginesFuelConsumpEq\4SRB\4SRB_400HP_G3408_Caterpillar.csv</t>
   </si>
 </sst>
 </file>
@@ -823,7 +826,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -874,6 +877,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1027,7 +1035,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1147,6 +1155,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -1488,10 +1502,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>208</v>
+        <v>191</v>
       </c>
       <c r="B5" t="s">
-        <v>209</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -1566,7 +1580,7 @@
         <v>7</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S1" s="11" t="s">
         <v>68</v>
@@ -1625,10 +1639,10 @@
         <v>110</v>
       </c>
       <c r="R2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="S2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1942,7 +1956,7 @@
         <v>47</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="F14" s="21" t="s">
         <v>29</v>
@@ -1965,7 +1979,7 @@
         <v>47</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="F15" s="21" t="s">
         <v>51</v>
@@ -1988,7 +2002,7 @@
         <v>47</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="F16" s="21" t="s">
         <v>51</v>
@@ -2011,7 +2025,7 @@
         <v>47</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="F17" s="21" t="s">
         <v>51</v>
@@ -2028,7 +2042,7 @@
         <v>47</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>47</v>
@@ -2051,7 +2065,7 @@
         <v>47</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>47</v>
@@ -2074,7 +2088,7 @@
         <v>47</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>47</v>
@@ -2103,13 +2117,13 @@
         <v>47</v>
       </c>
       <c r="E24" s="48" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="F24" s="48" t="s">
         <v>51</v>
       </c>
       <c r="G24" s="48" t="s">
-        <v>231</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2126,13 +2140,13 @@
         <v>47</v>
       </c>
       <c r="E25" s="48" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="F25" s="48" t="s">
         <v>51</v>
       </c>
       <c r="G25" s="48" t="s">
-        <v>232</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2149,13 +2163,13 @@
         <v>47</v>
       </c>
       <c r="E26" s="48" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="F26" s="48" t="s">
         <v>51</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>233</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2165,7 +2179,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4780323A-AA8D-4192-A121-B75F269C58B7}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -2409,7 +2423,7 @@
         <v>47</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="F14" s="21" t="s">
         <v>29</v>
@@ -2432,7 +2446,7 @@
         <v>47</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="F15" s="21" t="s">
         <v>51</v>
@@ -2455,150 +2469,12 @@
         <v>47</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="F16" s="21" t="s">
         <v>51</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="D18" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="48" t="s">
-        <v>230</v>
-      </c>
-      <c r="F18" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="48" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="D19" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="48" t="s">
-        <v>230</v>
-      </c>
-      <c r="F19" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="48" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="D20" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="48" t="s">
-        <v>230</v>
-      </c>
-      <c r="F20" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="G20" s="48" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="F22" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="G22" s="21" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="F23" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="G23" s="21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="F24" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="G24" s="21" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2709,7 +2585,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2733,10 +2609,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>226</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2757,33 +2633,25 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
         <v>22</v>
       </c>
     </row>
@@ -2940,7 +2808,7 @@
         <v>6</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>7</v>
@@ -3049,7 +2917,7 @@
         <v>35</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="R1" s="7" t="s">
         <v>43</v>
@@ -3114,7 +2982,7 @@
         <v>97</v>
       </c>
       <c r="S2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -3173,7 +3041,7 @@
         <v>97</v>
       </c>
       <c r="S3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3315,7 +3183,7 @@
         <v>35</v>
       </c>
       <c r="AJ1" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK1" s="7" t="s">
         <v>43</v>
@@ -3425,7 +3293,7 @@
         <v>134</v>
       </c>
       <c r="AH2" s="19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AI2" t="s">
         <v>11</v>
@@ -3437,7 +3305,7 @@
         <v>97</v>
       </c>
       <c r="AL2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.25">
@@ -3541,7 +3409,7 @@
         <v>134</v>
       </c>
       <c r="AH3" s="19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AI3" t="s">
         <v>11</v>
@@ -3553,7 +3421,7 @@
         <v>97</v>
       </c>
       <c r="AL3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3563,7 +3431,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF49C8AB-2E65-4CDC-84E1-9CD10D7B33D4}">
-  <dimension ref="A1:AK3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -3575,19 +3443,12 @@
     <col min="9" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="44" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="10" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
@@ -3630,77 +3491,20 @@
       <c r="N1" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="O1" s="35" t="s">
-        <v>113</v>
-      </c>
-      <c r="P1" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q1" s="35" t="s">
-        <v>115</v>
-      </c>
-      <c r="R1" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="S1" s="35" t="s">
-        <v>117</v>
-      </c>
-      <c r="T1" s="35" t="s">
-        <v>118</v>
-      </c>
-      <c r="U1" s="35" t="s">
-        <v>119</v>
-      </c>
-      <c r="V1" s="35" t="s">
-        <v>120</v>
-      </c>
-      <c r="W1" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="X1" s="27" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y1" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z1" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="AA1" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="AB1" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="AC1" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="AD1" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="AE1" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="AF1" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="AG1" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="AH1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="AI1" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="AJ1" s="7" t="s">
+      <c r="P1" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="Q1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="AK1" s="11" t="s">
+      <c r="R1" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -3743,77 +3547,20 @@
       <c r="N2">
         <v>1</v>
       </c>
-      <c r="O2" s="19">
-        <v>1</v>
-      </c>
-      <c r="P2" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="Q2" s="19">
-        <v>1</v>
-      </c>
-      <c r="R2" s="19">
-        <v>0.4</v>
-      </c>
-      <c r="S2" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="T2" s="19">
-        <v>0.6</v>
-      </c>
-      <c r="U2" s="19">
-        <v>1</v>
-      </c>
-      <c r="V2" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="W2" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="X2" s="31">
-        <v>2</v>
-      </c>
-      <c r="Y2" s="31">
-        <v>3</v>
-      </c>
-      <c r="Z2" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="AA2" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="AB2" s="31">
-        <v>2</v>
-      </c>
-      <c r="AC2" s="31">
-        <v>3</v>
-      </c>
-      <c r="AD2" s="31">
-        <v>2</v>
-      </c>
-      <c r="AE2" s="31">
-        <v>3</v>
-      </c>
-      <c r="AF2" s="31" t="s">
-        <v>134</v>
-      </c>
-      <c r="AG2" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="AH2" t="s">
+      <c r="O2" t="s">
         <v>11</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="P2" t="s">
         <v>111</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="Q2" t="s">
         <v>97</v>
       </c>
-      <c r="AK2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="R2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>47</v>
       </c>
@@ -3856,74 +3603,17 @@
       <c r="N3">
         <v>1</v>
       </c>
-      <c r="O3" s="19">
-        <v>1</v>
-      </c>
-      <c r="P3" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="Q3" s="19">
-        <v>1</v>
-      </c>
-      <c r="R3" s="19">
-        <v>0.4</v>
-      </c>
-      <c r="S3" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="T3" s="19">
-        <v>0.6</v>
-      </c>
-      <c r="U3" s="19">
-        <v>1</v>
-      </c>
-      <c r="V3" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="W3" s="31" t="b">
-        <v>0</v>
-      </c>
-      <c r="X3" s="31">
-        <v>2</v>
-      </c>
-      <c r="Y3" s="31">
-        <v>3</v>
-      </c>
-      <c r="Z3" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="AA3" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="AB3" s="31">
-        <v>2</v>
-      </c>
-      <c r="AC3" s="31">
-        <v>3</v>
-      </c>
-      <c r="AD3" s="31">
-        <v>2</v>
-      </c>
-      <c r="AE3" s="31">
-        <v>3</v>
-      </c>
-      <c r="AF3" s="31" t="s">
-        <v>134</v>
-      </c>
-      <c r="AG3" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="AH3" t="s">
+      <c r="O3" t="s">
         <v>11</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="P3" t="s">
         <v>111</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="Q3" t="s">
         <v>97</v>
       </c>
-      <c r="AK3" t="s">
-        <v>143</v>
+      <c r="R3" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3933,7 +3623,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -4005,7 +3695,7 @@
         <v>36</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="R1" s="11" t="s">
         <v>68</v>
@@ -4019,7 +3709,7 @@
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D2" s="6">
         <v>365</v>
@@ -4061,10 +3751,10 @@
         <v>52</v>
       </c>
       <c r="Q2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4075,7 +3765,7 @@
         <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D3" s="6">
         <v>365</v>
@@ -4117,66 +3807,10 @@
         <v>74</v>
       </c>
       <c r="Q3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" t="s">
-        <v>207</v>
-      </c>
-      <c r="C5" t="s">
-        <v>141</v>
-      </c>
-      <c r="D5" s="6">
-        <v>365</v>
-      </c>
-      <c r="E5" s="6">
-        <v>20</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0.02</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5" s="16">
-        <v>5</v>
-      </c>
-      <c r="J5" s="16">
-        <v>25</v>
-      </c>
-      <c r="K5" s="12">
-        <v>0</v>
-      </c>
-      <c r="L5" s="12">
-        <v>0.9</v>
-      </c>
-      <c r="M5" s="12">
-        <v>3</v>
-      </c>
-      <c r="N5" s="12">
-        <v>7</v>
-      </c>
-      <c r="O5" s="12">
-        <v>0.6</v>
-      </c>
-      <c r="P5" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>206</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -4215,37 +3849,37 @@
         <v>8</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>219</v>
+        <v>202</v>
       </c>
       <c r="F1" s="45" t="s">
+        <v>203</v>
+      </c>
+      <c r="G1" s="45" t="s">
         <v>220</v>
       </c>
-      <c r="G1" s="45" t="s">
-        <v>238</v>
-      </c>
       <c r="H1" s="45" t="s">
-        <v>221</v>
+        <v>204</v>
       </c>
       <c r="I1" s="45" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="J1" s="45" t="s">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="K1" s="45" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="L1" s="45" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="M1" s="45" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
       <c r="N1" s="45" t="s">
         <v>7</v>
@@ -4256,7 +3890,7 @@
         <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -4265,7 +3899,7 @@
         <v>8760</v>
       </c>
       <c r="E2" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="F2" s="47">
         <v>5.37</v>
@@ -4286,13 +3920,13 @@
         <v>48.24</v>
       </c>
       <c r="L2" t="s">
-        <v>228</v>
+        <v>211</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -4302,12 +3936,14 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFFCFF2C-DAB7-4E04-A795-0A279EB5D26F}">
-  <dimension ref="A1:BB2"/>
+  <dimension ref="A1:BD2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="47.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="8" width="16.140625" customWidth="1"/>
     <col min="9" max="9" width="12.28515625" customWidth="1"/>
     <col min="10" max="10" width="69.5703125" bestFit="1" customWidth="1"/>
@@ -4323,336 +3959,348 @@
     <col min="54" max="54" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" s="43" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:56" s="43" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="51" t="s">
+        <v>228</v>
+      </c>
+      <c r="D1" s="52" t="s">
+        <v>229</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="H1" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="J1" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="G1" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="H1" s="37" t="s">
+      <c r="K1" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="38" t="s">
+      <c r="L1" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="J1" s="38" t="s">
+      <c r="M1" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="O1" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="M1" s="39" t="s">
+      <c r="P1" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="Q1" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="O1" s="36" t="s">
+      <c r="R1" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="P1" s="37" t="s">
+      <c r="S1" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="Q1" s="37" t="s">
+      <c r="T1" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="U1" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="V1" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="T1" s="40" t="s">
+      <c r="W1" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="U1" s="40" t="s">
+      <c r="X1" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="Y1" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="AB1" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="Z1" s="41" t="s">
+      <c r="AC1" s="41" t="s">
+        <v>231</v>
+      </c>
+      <c r="AD1" s="41" t="s">
+        <v>232</v>
+      </c>
+      <c r="AE1" s="41" t="s">
         <v>171</v>
       </c>
-      <c r="AA1" s="41" t="s">
+      <c r="AF1" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="AB1" s="41" t="s">
+      <c r="AG1" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="AC1" s="41" t="s">
+      <c r="AH1" s="41" t="s">
+        <v>233</v>
+      </c>
+      <c r="AI1" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="AJ1" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="AD1" s="38" t="s">
+      <c r="AK1" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="AE1" s="18" t="s">
+      <c r="AL1" s="35" t="s">
+        <v>235</v>
+      </c>
+      <c r="AM1" s="35" t="s">
+        <v>236</v>
+      </c>
+      <c r="AN1" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="AF1" s="41" t="s">
+      <c r="AO1" s="41" t="s">
         <v>177</v>
       </c>
-      <c r="AG1" s="18" t="s">
+      <c r="AP1" s="41" t="s">
+        <v>237</v>
+      </c>
+      <c r="AQ1" s="41" t="s">
+        <v>238</v>
+      </c>
+      <c r="AR1" s="41" t="s">
         <v>178</v>
       </c>
-      <c r="AH1" s="41" t="s">
+      <c r="AS1" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="AI1" s="35" t="s">
+      <c r="AT1" s="42" t="s">
+        <v>239</v>
+      </c>
+      <c r="AU1" s="42" t="s">
+        <v>240</v>
+      </c>
+      <c r="AV1" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="AJ1" s="35" t="s">
+      <c r="AW1" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="AK1" s="35" t="s">
+      <c r="AX1" s="35" t="s">
+        <v>241</v>
+      </c>
+      <c r="AY1" s="35" t="s">
+        <v>242</v>
+      </c>
+      <c r="AZ1" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="AL1" s="35" t="s">
+      <c r="BA1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="BB1" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="BC1" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="AM1" s="41" t="s">
+      <c r="BD1" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
         <v>184</v>
       </c>
-      <c r="AN1" s="41" t="s">
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="E2" s="6">
+        <v>365</v>
+      </c>
+      <c r="F2" s="6">
+        <v>750</v>
+      </c>
+      <c r="G2" s="6">
+        <v>1E-10</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J2" t="s">
+        <v>243</v>
+      </c>
+      <c r="K2">
+        <v>0.7</v>
+      </c>
+      <c r="L2" t="s">
+        <v>244</v>
+      </c>
+      <c r="M2">
+        <v>0.35</v>
+      </c>
+      <c r="N2" t="s">
         <v>185</v>
       </c>
-      <c r="AO1" s="41" t="s">
+      <c r="O2" t="s">
+        <v>189</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="AP1" s="41" t="s">
-        <v>187</v>
-      </c>
-      <c r="AQ1" s="42" t="s">
-        <v>188</v>
-      </c>
-      <c r="AR1" s="42" t="s">
-        <v>189</v>
-      </c>
-      <c r="AS1" s="42" t="s">
-        <v>190</v>
-      </c>
-      <c r="AT1" s="42" t="s">
-        <v>191</v>
-      </c>
-      <c r="AU1" s="35" t="s">
-        <v>192</v>
-      </c>
-      <c r="AV1" s="35" t="s">
-        <v>193</v>
-      </c>
-      <c r="AW1" s="35" t="s">
-        <v>194</v>
-      </c>
-      <c r="AX1" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="AY1" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="AZ1" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="BA1" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="BB1" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C2" s="6">
-        <v>365</v>
-      </c>
-      <c r="D2" s="6">
-        <v>750</v>
-      </c>
-      <c r="E2" s="6">
-        <v>1E-10</v>
-      </c>
-      <c r="F2">
-        <v>600</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H2" t="s">
-        <v>202</v>
-      </c>
-      <c r="I2">
-        <v>0.7</v>
-      </c>
-      <c r="J2" t="s">
-        <v>203</v>
-      </c>
-      <c r="K2">
-        <v>0.35</v>
-      </c>
-      <c r="L2" t="s">
-        <v>198</v>
-      </c>
-      <c r="M2" t="s">
-        <v>204</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="P2">
-        <v>0.7</v>
-      </c>
-      <c r="Q2">
+      <c r="R2">
+        <v>0.9</v>
+      </c>
+      <c r="S2">
         <v>0.05</v>
       </c>
-      <c r="R2">
+      <c r="T2">
         <v>0.4</v>
       </c>
-      <c r="S2">
+      <c r="U2">
         <v>0.6</v>
       </c>
-      <c r="T2">
+      <c r="V2">
         <f>24*21</f>
         <v>504</v>
       </c>
-      <c r="U2">
+      <c r="W2">
         <f>24*7*6</f>
         <v>1008</v>
       </c>
-      <c r="V2">
+      <c r="X2">
         <v>300</v>
       </c>
-      <c r="W2">
+      <c r="Y2">
         <v>500</v>
       </c>
-      <c r="X2">
-        <f t="shared" ref="X2" si="0">60*15</f>
+      <c r="Z2">
+        <f t="shared" ref="Z2" si="0">60*15</f>
         <v>900</v>
       </c>
-      <c r="Y2">
-        <f t="shared" ref="Y2" si="1">ROUND(150*600/14.7,0)</f>
+      <c r="AA2">
+        <f t="shared" ref="AA2" si="1">ROUND(150*600/14.7,0)</f>
         <v>6122</v>
       </c>
-      <c r="Z2" s="20">
+      <c r="AB2" s="20">
         <v>1</v>
       </c>
-      <c r="AA2" s="20">
+      <c r="AC2" s="20">
         <v>0</v>
       </c>
-      <c r="AB2" s="20">
+      <c r="AD2" s="20">
         <v>4380</v>
       </c>
-      <c r="AC2" s="20">
+      <c r="AE2" s="20">
         <v>0.21634999999999999</v>
       </c>
-      <c r="AD2" t="b">
+      <c r="AF2" t="b">
         <v>1</v>
       </c>
-      <c r="AE2" s="20">
+      <c r="AG2" s="20">
         <v>1</v>
       </c>
-      <c r="AF2" s="20">
+      <c r="AH2" s="20">
         <v>0</v>
       </c>
-      <c r="AG2" s="20">
+      <c r="AI2" s="20">
         <v>4380</v>
       </c>
-      <c r="AH2" s="20">
+      <c r="AJ2" s="20">
         <v>8.3141000000000007E-2</v>
       </c>
-      <c r="AI2" s="19">
+      <c r="AK2" s="19">
         <v>1</v>
       </c>
-      <c r="AJ2" s="19">
+      <c r="AL2" s="19">
         <v>0</v>
       </c>
-      <c r="AK2" s="19">
+      <c r="AM2" s="19">
         <v>4380</v>
       </c>
-      <c r="AL2" s="19">
+      <c r="AN2" s="19">
         <v>0.47815999999999997</v>
       </c>
-      <c r="AM2" s="20">
+      <c r="AO2" s="20">
         <v>1</v>
       </c>
-      <c r="AN2" s="20">
+      <c r="AP2" s="20">
         <v>0</v>
       </c>
-      <c r="AO2" s="20">
+      <c r="AQ2" s="20">
         <v>2920</v>
       </c>
-      <c r="AP2" s="20">
+      <c r="AR2" s="20">
         <v>2.6738E-3</v>
       </c>
-      <c r="AQ2" s="44">
+      <c r="AS2" s="44">
         <v>1</v>
       </c>
-      <c r="AR2" s="44">
+      <c r="AT2" s="44">
         <v>0</v>
       </c>
-      <c r="AS2" s="44">
+      <c r="AU2" s="44">
         <v>4380</v>
       </c>
-      <c r="AT2" s="44">
+      <c r="AV2" s="44">
         <v>0.11268</v>
       </c>
-      <c r="AU2" s="19">
+      <c r="AW2" s="19">
         <v>1</v>
       </c>
-      <c r="AV2" s="19">
+      <c r="AX2" s="19">
         <v>0</v>
       </c>
-      <c r="AW2" s="19">
+      <c r="AY2" s="19">
         <v>2920</v>
       </c>
-      <c r="AX2" s="19">
+      <c r="AZ2" s="19">
         <v>2.7855000000000002E-3</v>
       </c>
-      <c r="AY2" t="s">
-        <v>200</v>
-      </c>
-      <c r="AZ2" t="s">
+      <c r="BA2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BB2" t="s">
         <v>111</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BC2" t="s">
         <v>111</v>
       </c>
-      <c r="BB2" t="s">
-        <v>201</v>
+      <c r="BD2" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -4667,7 +4315,7 @@
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" customWidth="1"/>
@@ -4696,7 +4344,7 @@
         <v>8</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>94</v>
@@ -4720,7 +4368,7 @@
         <v>81</v>
       </c>
       <c r="L1" s="24" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="M1" s="25" t="s">
         <v>82</v>
@@ -4741,46 +4389,46 @@
         <v>87</v>
       </c>
       <c r="S1" s="25" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
       <c r="T1" s="25" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="U1" s="25" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="V1" s="26" t="s">
-        <v>213</v>
+        <v>196</v>
       </c>
       <c r="W1" s="26" t="s">
-        <v>214</v>
+        <v>197</v>
       </c>
       <c r="X1" s="26" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="Y1" s="27" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="Z1" s="27" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="AA1" s="27" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="AB1" s="27" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="AC1" s="27" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="AD1" s="27" t="s">
-        <v>236</v>
+        <v>219</v>
       </c>
       <c r="AE1" s="49" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="AF1" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG1" s="7" t="s">
         <v>68</v>
@@ -4878,13 +4526,13 @@
         <v>5000</v>
       </c>
       <c r="AE2" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AG2" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
@@ -4922,7 +4570,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" s="29">
         <v>0</v>
@@ -4979,13 +4627,13 @@
         <v>5000</v>
       </c>
       <c r="AE3" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AG3" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>